<commit_message>
feat: Incremental & streaming quotes, v3.0.0
Signed-off-by: Dave Skender <8432125+DaveSkender@users.noreply.github.com>
Co-authored-by: JGronholz <17935969+JGronholz@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/indicators/a-d/Adx/Adx.Calc.xlsx
+++ b/tests/indicators/a-d/Adx/Adx.Calc.xlsx
@@ -1,26 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <fileSharing readOnlyRecommended="1"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D1D8B8F-9F53-4B0A-A856-4006463BEA60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3415FB2C-712A-4184-A87B-956C4B37A34C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36480" yWindow="0" windowWidth="28800" windowHeight="21690" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ADX" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -607,7 +598,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1544,22 +1535,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y503"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="9" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" customWidth="1"/>
-    <col min="12" max="16" width="9.140625" style="7"/>
-    <col min="17" max="17" width="3.7109375" customWidth="1"/>
-    <col min="18" max="18" width="8.140625" style="5" customWidth="1"/>
-    <col min="19" max="21" width="9.140625" style="7"/>
-    <col min="23" max="23" width="8.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="9.140625" style="7"/>
+    <col min="9" max="9" width="9.1796875" customWidth="1"/>
+    <col min="12" max="16" width="9.1796875" style="7"/>
+    <col min="17" max="17" width="3.7265625" customWidth="1"/>
+    <col min="18" max="18" width="8.1796875" style="5" customWidth="1"/>
+    <col min="19" max="21" width="9.1796875" style="7"/>
+    <col min="23" max="23" width="8.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="9.1796875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>20</v>
       </c>
@@ -1630,7 +1621,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
         <v>0</v>
       </c>
@@ -1669,7 +1660,7 @@
       <c r="X2" s="6"/>
       <c r="Y2" s="6"/>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -1717,7 +1708,7 @@
       <c r="X3" s="6"/>
       <c r="Y3" s="6"/>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>2</v>
       </c>
@@ -1765,7 +1756,7 @@
       <c r="X4" s="6"/>
       <c r="Y4" s="6"/>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>3</v>
       </c>
@@ -1813,7 +1804,7 @@
       <c r="X5" s="6"/>
       <c r="Y5" s="6"/>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>4</v>
       </c>
@@ -1861,7 +1852,7 @@
       <c r="X6" s="6"/>
       <c r="Y6" s="6"/>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>5</v>
       </c>
@@ -1909,7 +1900,7 @@
       <c r="X7" s="6"/>
       <c r="Y7" s="6"/>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>6</v>
       </c>
@@ -1957,7 +1948,7 @@
       <c r="X8" s="6"/>
       <c r="Y8" s="6"/>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>7</v>
       </c>
@@ -2005,7 +1996,7 @@
       <c r="X9" s="6"/>
       <c r="Y9" s="6"/>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>8</v>
       </c>
@@ -2053,7 +2044,7 @@
       <c r="X10" s="6"/>
       <c r="Y10" s="6"/>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>9</v>
       </c>
@@ -2101,7 +2092,7 @@
       <c r="X11" s="6"/>
       <c r="Y11" s="6"/>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>10</v>
       </c>
@@ -2149,7 +2140,7 @@
       <c r="X12" s="6"/>
       <c r="Y12" s="6"/>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>11</v>
       </c>
@@ -2197,7 +2188,7 @@
       <c r="X13" s="6"/>
       <c r="Y13" s="6"/>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
         <v>12</v>
       </c>
@@ -2245,7 +2236,7 @@
       <c r="X14" s="6"/>
       <c r="Y14" s="6"/>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
         <v>13</v>
       </c>
@@ -2293,7 +2284,7 @@
       <c r="X15" s="6"/>
       <c r="Y15" s="6"/>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
         <v>14</v>
       </c>
@@ -2363,7 +2354,7 @@
       <c r="X16" s="6"/>
       <c r="Y16" s="6"/>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
         <v>15</v>
       </c>
@@ -2433,7 +2424,7 @@
       <c r="X17" s="6"/>
       <c r="Y17" s="6"/>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
         <v>16</v>
       </c>
@@ -2503,7 +2494,7 @@
       <c r="X18" s="6"/>
       <c r="Y18" s="6"/>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
         <v>17</v>
       </c>
@@ -2573,7 +2564,7 @@
       <c r="X19" s="6"/>
       <c r="Y19" s="6"/>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
         <v>18</v>
       </c>
@@ -2643,7 +2634,7 @@
       <c r="X20" s="6"/>
       <c r="Y20" s="6"/>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A21" s="4">
         <v>19</v>
       </c>
@@ -2691,7 +2682,7 @@
         <f>100*testdata[[#This Row],[-DM14]]/testdata[[#This Row],[TR14]]</f>
         <v>25.012425579421205</v>
       </c>
-      <c r="N21" s="6">
+      <c r="N21" s="11">
         <f>100*ABS(testdata[[#This Row],[+DI14]]-testdata[[#This Row],[-DI14]])/(testdata[[#This Row],[+DI14]]+testdata[[#This Row],[-DI14]])</f>
         <v>8.6351139279442961</v>
       </c>
@@ -2713,7 +2704,7 @@
       <c r="X21" s="11"/>
       <c r="Y21" s="11"/>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A22" s="4">
         <v>20</v>
       </c>
@@ -2783,7 +2774,7 @@
       <c r="X22" s="6"/>
       <c r="Y22" s="6"/>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A23" s="4">
         <v>21</v>
       </c>
@@ -2853,7 +2844,7 @@
       <c r="X23" s="6"/>
       <c r="Y23" s="6"/>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A24" s="4">
         <v>22</v>
       </c>
@@ -2923,7 +2914,7 @@
       <c r="X24" s="6"/>
       <c r="Y24" s="6"/>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A25" s="4">
         <v>23</v>
       </c>
@@ -2993,7 +2984,7 @@
       <c r="X25" s="6"/>
       <c r="Y25" s="6"/>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A26" s="4">
         <v>24</v>
       </c>
@@ -3063,7 +3054,7 @@
       <c r="X26" s="6"/>
       <c r="Y26" s="6"/>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A27" s="4">
         <v>25</v>
       </c>
@@ -3133,7 +3124,7 @@
       <c r="X27" s="6"/>
       <c r="Y27" s="6"/>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A28" s="4">
         <v>26</v>
       </c>
@@ -3203,7 +3194,7 @@
       <c r="X28" s="6"/>
       <c r="Y28" s="6"/>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A29" s="4">
         <v>27</v>
       </c>
@@ -3280,7 +3271,7 @@
       </c>
       <c r="Y29" s="13"/>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A30" s="4">
         <v>28</v>
       </c>
@@ -3357,7 +3348,7 @@
       </c>
       <c r="Y30" s="6"/>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A31" s="4">
         <v>29</v>
       </c>
@@ -3405,7 +3396,7 @@
         <f>100*testdata[[#This Row],[-DM14]]/testdata[[#This Row],[TR14]]</f>
         <v>14.165829841353299</v>
       </c>
-      <c r="N31" s="6">
+      <c r="N31" s="11">
         <f>100*ABS(testdata[[#This Row],[+DI14]]-testdata[[#This Row],[-DI14]])/(testdata[[#This Row],[+DI14]]+testdata[[#This Row],[-DI14]])</f>
         <v>45.659962116806589</v>
       </c>
@@ -3434,7 +3425,7 @@
       </c>
       <c r="Y31" s="11"/>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A32" s="4">
         <v>30</v>
       </c>
@@ -3511,7 +3502,7 @@
       </c>
       <c r="Y32" s="6"/>
     </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A33" s="4">
         <v>31</v>
       </c>
@@ -3588,7 +3579,7 @@
       </c>
       <c r="Y33" s="6"/>
     </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A34" s="4">
         <v>32</v>
       </c>
@@ -3665,7 +3656,7 @@
       </c>
       <c r="Y34" s="6"/>
     </row>
-    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A35" s="4">
         <v>33</v>
       </c>
@@ -3742,7 +3733,7 @@
       </c>
       <c r="Y35" s="6"/>
     </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A36" s="4">
         <v>34</v>
       </c>
@@ -3819,7 +3810,7 @@
       </c>
       <c r="Y36" s="6"/>
     </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A37" s="4">
         <v>35</v>
       </c>
@@ -3896,7 +3887,7 @@
       </c>
       <c r="Y37" s="6"/>
     </row>
-    <row r="38" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A38" s="4">
         <v>36</v>
       </c>
@@ -3973,7 +3964,7 @@
       </c>
       <c r="Y38" s="6"/>
     </row>
-    <row r="39" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A39" s="4">
         <v>37</v>
       </c>
@@ -4050,7 +4041,7 @@
       </c>
       <c r="Y39" s="6"/>
     </row>
-    <row r="40" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A40" s="4">
         <v>38</v>
       </c>
@@ -4127,7 +4118,7 @@
       </c>
       <c r="Y40" s="6"/>
     </row>
-    <row r="41" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A41" s="4">
         <v>39</v>
       </c>
@@ -4204,7 +4195,7 @@
       </c>
       <c r="Y41" s="6"/>
     </row>
-    <row r="42" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A42" s="4">
         <v>40</v>
       </c>
@@ -4286,7 +4277,7 @@
         <v>29.1061924422517</v>
       </c>
     </row>
-    <row r="43" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A43" s="4">
         <v>41</v>
       </c>
@@ -4368,7 +4359,7 @@
         <v>30.612091066317898</v>
       </c>
     </row>
-    <row r="44" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A44" s="4">
         <v>42</v>
       </c>
@@ -4450,7 +4441,7 @@
         <v>31.742940902605799</v>
       </c>
     </row>
-    <row r="45" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A45" s="4">
         <v>43</v>
       </c>
@@ -4532,7 +4523,7 @@
         <v>32.910704164193803</v>
       </c>
     </row>
-    <row r="46" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A46" s="4">
         <v>44</v>
       </c>
@@ -4614,7 +4605,7 @@
         <v>33.800668233057998</v>
       </c>
     </row>
-    <row r="47" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A47" s="4">
         <v>45</v>
       </c>
@@ -4696,7 +4687,7 @@
         <v>34.282530871755498</v>
       </c>
     </row>
-    <row r="48" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A48" s="4">
         <v>46</v>
       </c>
@@ -4778,7 +4769,7 @@
         <v>35.203773847973203</v>
       </c>
     </row>
-    <row r="49" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A49" s="4">
         <v>47</v>
       </c>
@@ -4860,7 +4851,7 @@
         <v>36.059213754461098</v>
       </c>
     </row>
-    <row r="50" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A50" s="4">
         <v>48</v>
       </c>
@@ -4942,7 +4933,7 @@
         <v>36.365003212984099</v>
       </c>
     </row>
-    <row r="51" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A51" s="4">
         <v>49</v>
       </c>
@@ -5024,7 +5015,7 @@
         <v>37.142611710382397</v>
       </c>
     </row>
-    <row r="52" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A52" s="4">
         <v>50</v>
       </c>
@@ -5106,7 +5097,7 @@
         <v>37.952532158976197</v>
       </c>
     </row>
-    <row r="53" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A53" s="4">
         <v>51</v>
       </c>
@@ -5188,7 +5179,7 @@
         <v>38.4561721826583</v>
       </c>
     </row>
-    <row r="54" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A54" s="4">
         <v>52</v>
       </c>
@@ -5270,7 +5261,7 @@
         <v>39.044472480502797</v>
       </c>
     </row>
-    <row r="55" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A55" s="4">
         <v>53</v>
       </c>
@@ -5352,7 +5343,7 @@
         <v>38.805876785297102</v>
       </c>
     </row>
-    <row r="56" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A56" s="4">
         <v>54</v>
       </c>
@@ -5434,7 +5425,7 @@
         <v>38.471016752236899</v>
       </c>
     </row>
-    <row r="57" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A57" s="4">
         <v>55</v>
       </c>
@@ -5516,7 +5507,7 @@
         <v>37.4997691385419</v>
       </c>
     </row>
-    <row r="58" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A58" s="4">
         <v>56</v>
       </c>
@@ -5598,7 +5589,7 @@
         <v>36.665467018523003</v>
       </c>
     </row>
-    <row r="59" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A59" s="4">
         <v>57</v>
       </c>
@@ -5680,7 +5671,7 @@
         <v>36.079144579880399</v>
       </c>
     </row>
-    <row r="60" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A60" s="4">
         <v>58</v>
       </c>
@@ -5762,7 +5753,7 @@
         <v>34.551715527415404</v>
       </c>
     </row>
-    <row r="61" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A61" s="4">
         <v>59</v>
       </c>
@@ -5844,7 +5835,7 @@
         <v>33.344820747917403</v>
       </c>
     </row>
-    <row r="62" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A62" s="4">
         <v>60</v>
       </c>
@@ -5926,7 +5917,7 @@
         <v>32.366541473105897</v>
       </c>
     </row>
-    <row r="63" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A63" s="4">
         <v>61</v>
       </c>
@@ -6008,7 +5999,7 @@
         <v>30.914364787662802</v>
       </c>
     </row>
-    <row r="64" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A64" s="4">
         <v>62</v>
       </c>
@@ -6090,7 +6081,7 @@
         <v>30.357705712508601</v>
       </c>
     </row>
-    <row r="65" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A65" s="4">
         <v>63</v>
       </c>
@@ -6172,7 +6163,7 @@
         <v>29.840807999865401</v>
       </c>
     </row>
-    <row r="66" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A66" s="4">
         <v>64</v>
       </c>
@@ -6254,7 +6245,7 @@
         <v>29.172918215714301</v>
       </c>
     </row>
-    <row r="67" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A67" s="4">
         <v>65</v>
       </c>
@@ -6336,7 +6327,7 @@
         <v>28.1491072195229</v>
       </c>
     </row>
-    <row r="68" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A68" s="4">
         <v>66</v>
       </c>
@@ -6418,7 +6409,7 @@
         <v>26.504759350980599</v>
       </c>
     </row>
-    <row r="69" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A69" s="4">
         <v>67</v>
       </c>
@@ -6500,7 +6491,7 @@
         <v>25.231445672096498</v>
       </c>
     </row>
-    <row r="70" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A70" s="4">
         <v>68</v>
       </c>
@@ -6582,7 +6573,7 @@
         <v>23.7548435583547</v>
       </c>
     </row>
-    <row r="71" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A71" s="4">
         <v>69</v>
       </c>
@@ -6664,7 +6655,7 @@
         <v>22.5885590108646</v>
       </c>
     </row>
-    <row r="72" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A72" s="4">
         <v>70</v>
       </c>
@@ -6746,7 +6737,7 @@
         <v>22.295802015566402</v>
       </c>
     </row>
-    <row r="73" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A73" s="4">
         <v>71</v>
       </c>
@@ -6828,7 +6819,7 @@
         <v>21.349036701747899</v>
       </c>
     </row>
-    <row r="74" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A74" s="4">
         <v>72</v>
       </c>
@@ -6910,7 +6901,7 @@
         <v>20.4698974817737</v>
       </c>
     </row>
-    <row r="75" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A75" s="4">
         <v>73</v>
       </c>
@@ -6992,7 +6983,7 @@
         <v>19.577440110008901</v>
       </c>
     </row>
-    <row r="76" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A76" s="4">
         <v>74</v>
       </c>
@@ -7074,7 +7065,7 @@
         <v>18.364523548171501</v>
       </c>
     </row>
-    <row r="77" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A77" s="4">
         <v>75</v>
       </c>
@@ -7156,7 +7147,7 @@
         <v>17.4385494803442</v>
       </c>
     </row>
-    <row r="78" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A78" s="4">
         <v>76</v>
       </c>
@@ -7238,7 +7229,7 @@
         <v>17.329884510539799</v>
       </c>
     </row>
-    <row r="79" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A79" s="4">
         <v>77</v>
       </c>
@@ -7320,7 +7311,7 @@
         <v>17.4648063151473</v>
       </c>
     </row>
-    <row r="80" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A80" s="4">
         <v>78</v>
       </c>
@@ -7402,7 +7393,7 @@
         <v>17.682948149028899</v>
       </c>
     </row>
-    <row r="81" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A81" s="4">
         <v>79</v>
       </c>
@@ -7484,7 +7475,7 @@
         <v>17.7100214417076</v>
       </c>
     </row>
-    <row r="82" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A82" s="4">
         <v>80</v>
       </c>
@@ -7566,7 +7557,7 @@
         <v>17.799489278081499</v>
       </c>
     </row>
-    <row r="83" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A83" s="4">
         <v>81</v>
       </c>
@@ -7648,7 +7639,7 @@
         <v>17.915875466956699</v>
       </c>
     </row>
-    <row r="84" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A84" s="4">
         <v>82</v>
       </c>
@@ -7730,7 +7721,7 @@
         <v>18.023948356626502</v>
       </c>
     </row>
-    <row r="85" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A85" s="4">
         <v>83</v>
       </c>
@@ -7812,7 +7803,7 @@
         <v>18.1939708200286</v>
       </c>
     </row>
-    <row r="86" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A86" s="4">
         <v>84</v>
       </c>
@@ -7894,7 +7885,7 @@
         <v>18.333775819821199</v>
       </c>
     </row>
-    <row r="87" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A87" s="4">
         <v>85</v>
       </c>
@@ -7976,7 +7967,7 @@
         <v>18.729992570185601</v>
       </c>
     </row>
-    <row r="88" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A88" s="4">
         <v>86</v>
       </c>
@@ -8058,7 +8049,7 @@
         <v>18.943293212509801</v>
       </c>
     </row>
-    <row r="89" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A89" s="4">
         <v>87</v>
       </c>
@@ -8140,7 +8131,7 @@
         <v>18.845526482244999</v>
       </c>
     </row>
-    <row r="90" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A90" s="4">
         <v>88</v>
       </c>
@@ -8222,7 +8213,7 @@
         <v>18.754743089856301</v>
       </c>
     </row>
-    <row r="91" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A91" s="4">
         <v>89</v>
       </c>
@@ -8304,7 +8295,7 @@
         <v>18.760152884100101</v>
       </c>
     </row>
-    <row r="92" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A92" s="4">
         <v>90</v>
       </c>
@@ -8386,7 +8377,7 @@
         <v>19.1669628391214</v>
       </c>
     </row>
-    <row r="93" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A93" s="4">
         <v>91</v>
       </c>
@@ -8468,7 +8459,7 @@
         <v>20.081985790329501</v>
       </c>
     </row>
-    <row r="94" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A94" s="4">
         <v>92</v>
       </c>
@@ -8550,7 +8541,7 @@
         <v>20.836070292675601</v>
       </c>
     </row>
-    <row r="95" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A95" s="4">
         <v>93</v>
       </c>
@@ -8632,7 +8623,7 @@
         <v>21.073811681227099</v>
       </c>
     </row>
-    <row r="96" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A96" s="4">
         <v>94</v>
       </c>
@@ -8714,7 +8705,7 @@
         <v>21.455839944231698</v>
       </c>
     </row>
-    <row r="97" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A97" s="4">
         <v>95</v>
       </c>
@@ -8796,7 +8787,7 @@
         <v>21.2716280780853</v>
       </c>
     </row>
-    <row r="98" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A98" s="4">
         <v>96</v>
       </c>
@@ -8878,7 +8869,7 @@
         <v>20.5940638953319</v>
       </c>
     </row>
-    <row r="99" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A99" s="4">
         <v>97</v>
       </c>
@@ -8960,7 +8951,7 @@
         <v>20.167656670205499</v>
       </c>
     </row>
-    <row r="100" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A100" s="4">
         <v>98</v>
       </c>
@@ -9042,7 +9033,7 @@
         <v>20.199714171617</v>
       </c>
     </row>
-    <row r="101" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A101" s="4">
         <v>99</v>
       </c>
@@ -9124,7 +9115,7 @@
         <v>20.696337137899501</v>
       </c>
     </row>
-    <row r="102" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A102" s="4">
         <v>100</v>
       </c>
@@ -9206,7 +9197,7 @@
         <v>21.245861567937698</v>
       </c>
     </row>
-    <row r="103" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A103" s="4">
         <v>101</v>
       </c>
@@ -9288,7 +9279,7 @@
         <v>21.6262416569778</v>
       </c>
     </row>
-    <row r="104" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A104" s="4">
         <v>102</v>
       </c>
@@ -9370,7 +9361,7 @@
         <v>21.085307012226501</v>
       </c>
     </row>
-    <row r="105" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A105" s="4">
         <v>103</v>
       </c>
@@ -9452,7 +9443,7 @@
         <v>21.049995180387899</v>
       </c>
     </row>
-    <row r="106" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A106" s="4">
         <v>104</v>
       </c>
@@ -9534,7 +9525,7 @@
         <v>21.672467470452801</v>
       </c>
     </row>
-    <row r="107" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A107" s="4">
         <v>105</v>
       </c>
@@ -9616,7 +9607,7 @@
         <v>22.330384769091701</v>
       </c>
     </row>
-    <row r="108" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A108" s="4">
         <v>106</v>
       </c>
@@ -9698,7 +9689,7 @@
         <v>22.191305661936902</v>
       </c>
     </row>
-    <row r="109" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A109" s="4">
         <v>107</v>
       </c>
@@ -9780,7 +9771,7 @@
         <v>22.017220872573901</v>
       </c>
     </row>
-    <row r="110" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A110" s="4">
         <v>108</v>
       </c>
@@ -9862,7 +9853,7 @@
         <v>21.448871413869199</v>
       </c>
     </row>
-    <row r="111" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A111" s="4">
         <v>109</v>
       </c>
@@ -9944,7 +9935,7 @@
         <v>20.1916776939816</v>
       </c>
     </row>
-    <row r="112" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A112" s="4">
         <v>110</v>
       </c>
@@ -10026,7 +10017,7 @@
         <v>19.208650730890302</v>
       </c>
     </row>
-    <row r="113" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A113" s="4">
         <v>111</v>
       </c>
@@ -10108,7 +10099,7 @@
         <v>18.876123557151701</v>
       </c>
     </row>
-    <row r="114" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A114" s="4">
         <v>112</v>
       </c>
@@ -10190,7 +10181,7 @@
         <v>18.8323775209107</v>
       </c>
     </row>
-    <row r="115" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A115" s="4">
         <v>113</v>
       </c>
@@ -10272,7 +10263,7 @@
         <v>18.384938741852299</v>
       </c>
     </row>
-    <row r="116" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A116" s="4">
         <v>114</v>
       </c>
@@ -10354,7 +10345,7 @@
         <v>17.880924714904499</v>
       </c>
     </row>
-    <row r="117" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A117" s="4">
         <v>115</v>
       </c>
@@ -10436,7 +10427,7 @@
         <v>17.8257912322909</v>
       </c>
     </row>
-    <row r="118" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A118" s="4">
         <v>116</v>
       </c>
@@ -10518,7 +10509,7 @@
         <v>18.021104841539</v>
       </c>
     </row>
-    <row r="119" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A119" s="4">
         <v>117</v>
       </c>
@@ -10600,7 +10591,7 @@
         <v>18.204445089235399</v>
       </c>
     </row>
-    <row r="120" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A120" s="4">
         <v>118</v>
       </c>
@@ -10682,7 +10673,7 @@
         <v>18.374689604953399</v>
       </c>
     </row>
-    <row r="121" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A121" s="4">
         <v>119</v>
       </c>
@@ -10764,7 +10755,7 @@
         <v>18.1374786511679</v>
       </c>
     </row>
-    <row r="122" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A122" s="4">
         <v>120</v>
       </c>
@@ -10846,7 +10837,7 @@
         <v>18.105568195448399</v>
       </c>
     </row>
-    <row r="123" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A123" s="4">
         <v>121</v>
       </c>
@@ -10928,7 +10919,7 @@
         <v>17.760763803450999</v>
       </c>
     </row>
-    <row r="124" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A124" s="4">
         <v>122</v>
       </c>
@@ -11010,7 +11001,7 @@
         <v>16.7507030014878</v>
       </c>
     </row>
-    <row r="125" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A125" s="4">
         <v>123</v>
       </c>
@@ -11092,7 +11083,7 @@
         <v>16.542459502739199</v>
       </c>
     </row>
-    <row r="126" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A126" s="4">
         <v>124</v>
       </c>
@@ -11174,7 +11165,7 @@
         <v>16.767764871704099</v>
       </c>
     </row>
-    <row r="127" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A127" s="4">
         <v>125</v>
       </c>
@@ -11256,7 +11247,7 @@
         <v>16.556801427059099</v>
       </c>
     </row>
-    <row r="128" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A128" s="4">
         <v>126</v>
       </c>
@@ -11338,7 +11329,7 @@
         <v>16.113631331442001</v>
       </c>
     </row>
-    <row r="129" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A129" s="4">
         <v>127</v>
       </c>
@@ -11420,7 +11411,7 @@
         <v>16.120742708005</v>
       </c>
     </row>
-    <row r="130" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A130" s="4">
         <v>128</v>
       </c>
@@ -11502,7 +11493,7 @@
         <v>16.6599037100797</v>
       </c>
     </row>
-    <row r="131" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A131" s="4">
         <v>129</v>
       </c>
@@ -11584,7 +11575,7 @@
         <v>16.705822336562999</v>
       </c>
     </row>
-    <row r="132" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A132" s="4">
         <v>130</v>
       </c>
@@ -11666,7 +11657,7 @@
         <v>16.7628409089901</v>
       </c>
     </row>
-    <row r="133" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A133" s="4">
         <v>131</v>
       </c>
@@ -11748,7 +11739,7 @@
         <v>16.150396947228401</v>
       </c>
     </row>
-    <row r="134" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A134" s="4">
         <v>132</v>
       </c>
@@ -11830,7 +11821,7 @@
         <v>15.3720936341465</v>
       </c>
     </row>
-    <row r="135" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A135" s="4">
         <v>133</v>
       </c>
@@ -11912,7 +11903,7 @@
         <v>15.207804271541301</v>
       </c>
     </row>
-    <row r="136" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A136" s="4">
         <v>134</v>
       </c>
@@ -11994,7 +11985,7 @@
         <v>14.607823509938299</v>
       </c>
     </row>
-    <row r="137" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A137" s="4">
         <v>135</v>
       </c>
@@ -12076,7 +12067,7 @@
         <v>13.6711197999911</v>
       </c>
     </row>
-    <row r="138" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A138" s="4">
         <v>136</v>
       </c>
@@ -12158,7 +12149,7 @@
         <v>13.937102595633201</v>
       </c>
     </row>
-    <row r="139" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A139" s="4">
         <v>137</v>
       </c>
@@ -12240,7 +12231,7 @@
         <v>14.305698275808799</v>
       </c>
     </row>
-    <row r="140" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A140" s="4">
         <v>138</v>
       </c>
@@ -12322,7 +12313,7 @@
         <v>14.243953693353401</v>
       </c>
     </row>
-    <row r="141" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A141" s="4">
         <v>139</v>
       </c>
@@ -12404,7 +12395,7 @@
         <v>14.366568041736301</v>
       </c>
     </row>
-    <row r="142" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A142" s="4">
         <v>140</v>
       </c>
@@ -12486,7 +12477,7 @@
         <v>15.1203531340515</v>
       </c>
     </row>
-    <row r="143" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A143" s="4">
         <v>141</v>
       </c>
@@ -12568,7 +12559,7 @@
         <v>15.691984664705901</v>
       </c>
     </row>
-    <row r="144" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A144" s="4">
         <v>142</v>
       </c>
@@ -12650,7 +12641,7 @@
         <v>15.3449938541245</v>
       </c>
     </row>
-    <row r="145" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A145" s="4">
         <v>143</v>
       </c>
@@ -12732,7 +12723,7 @@
         <v>15.285300670218</v>
       </c>
     </row>
-    <row r="146" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A146" s="4">
         <v>144</v>
       </c>
@@ -12814,7 +12805,7 @@
         <v>14.727913284457699</v>
       </c>
     </row>
-    <row r="147" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A147" s="4">
         <v>145</v>
       </c>
@@ -12896,7 +12887,7 @@
         <v>14.090988831051201</v>
       </c>
     </row>
-    <row r="148" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A148" s="4">
         <v>146</v>
       </c>
@@ -12978,7 +12969,7 @@
         <v>13.561939402961</v>
       </c>
     </row>
-    <row r="149" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A149" s="4">
         <v>147</v>
       </c>
@@ -13060,7 +13051,7 @@
         <v>13.070679219734499</v>
       </c>
     </row>
-    <row r="150" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A150" s="4">
         <v>148</v>
       </c>
@@ -13142,7 +13133,7 @@
         <v>12.5772595112294</v>
       </c>
     </row>
-    <row r="151" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A151" s="4">
         <v>149</v>
       </c>
@@ -13224,7 +13215,7 @@
         <v>12.5596040027716</v>
       </c>
     </row>
-    <row r="152" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A152" s="4">
         <v>150</v>
       </c>
@@ -13306,7 +13297,7 @@
         <v>13.110921462571101</v>
       </c>
     </row>
-    <row r="153" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A153" s="4">
         <v>151</v>
       </c>
@@ -13388,7 +13379,7 @@
         <v>13.062343953195899</v>
       </c>
     </row>
-    <row r="154" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A154" s="4">
         <v>152</v>
       </c>
@@ -13470,7 +13461,7 @@
         <v>13.252946001101799</v>
       </c>
     </row>
-    <row r="155" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A155" s="4">
         <v>153</v>
       </c>
@@ -13552,7 +13543,7 @@
         <v>13.692593498654</v>
       </c>
     </row>
-    <row r="156" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A156" s="4">
         <v>154</v>
       </c>
@@ -13634,7 +13625,7 @@
         <v>13.699636441906801</v>
       </c>
     </row>
-    <row r="157" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A157" s="4">
         <v>155</v>
       </c>
@@ -13716,7 +13707,7 @@
         <v>13.1356829936324</v>
       </c>
     </row>
-    <row r="158" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A158" s="4">
         <v>156</v>
       </c>
@@ -13798,7 +13789,7 @@
         <v>12.8108158536141</v>
       </c>
     </row>
-    <row r="159" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A159" s="4">
         <v>157</v>
       </c>
@@ -13880,7 +13871,7 @@
         <v>12.816410100620899</v>
       </c>
     </row>
-    <row r="160" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A160" s="4">
         <v>158</v>
       </c>
@@ -13962,7 +13953,7 @@
         <v>13.044485021236101</v>
       </c>
     </row>
-    <row r="161" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A161" s="4">
         <v>159</v>
       </c>
@@ -14044,7 +14035,7 @@
         <v>13.1763539087168</v>
       </c>
     </row>
-    <row r="162" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A162" s="4">
         <v>160</v>
       </c>
@@ -14126,7 +14117,7 @@
         <v>12.479310573888</v>
       </c>
     </row>
-    <row r="163" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A163" s="4">
         <v>161</v>
       </c>
@@ -14208,7 +14199,7 @@
         <v>12.0434436761443</v>
       </c>
     </row>
-    <row r="164" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A164" s="4">
         <v>162</v>
       </c>
@@ -14290,7 +14281,7 @@
         <v>11.7950640075442</v>
       </c>
     </row>
-    <row r="165" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A165" s="4">
         <v>163</v>
       </c>
@@ -14372,7 +14363,7 @@
         <v>11.8679599910823</v>
       </c>
     </row>
-    <row r="166" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A166" s="4">
         <v>164</v>
       </c>
@@ -14454,7 +14445,7 @@
         <v>11.5901761420778</v>
       </c>
     </row>
-    <row r="167" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A167" s="4">
         <v>165</v>
       </c>
@@ -14536,7 +14527,7 @@
         <v>11.895316982337601</v>
       </c>
     </row>
-    <row r="168" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A168" s="4">
         <v>166</v>
       </c>
@@ -14618,7 +14609,7 @@
         <v>11.7665845155101</v>
       </c>
     </row>
-    <row r="169" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A169" s="4">
         <v>167</v>
       </c>
@@ -14700,7 +14691,7 @@
         <v>11.453332262058799</v>
       </c>
     </row>
-    <row r="170" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A170" s="4">
         <v>168</v>
       </c>
@@ -14782,7 +14773,7 @@
         <v>11.386578842492</v>
       </c>
     </row>
-    <row r="171" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A171" s="4">
         <v>169</v>
       </c>
@@ -14864,7 +14855,7 @@
         <v>11.3865920698675</v>
       </c>
     </row>
-    <row r="172" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A172" s="4">
         <v>170</v>
       </c>
@@ -14946,7 +14937,7 @@
         <v>11.530429165428901</v>
       </c>
     </row>
-    <row r="173" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A173" s="4">
         <v>171</v>
       </c>
@@ -15028,7 +15019,7 @@
         <v>11.8785112450217</v>
       </c>
     </row>
-    <row r="174" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A174" s="4">
         <v>172</v>
       </c>
@@ -15110,7 +15101,7 @@
         <v>12.316903208731601</v>
       </c>
     </row>
-    <row r="175" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A175" s="4">
         <v>173</v>
       </c>
@@ -15192,7 +15183,7 @@
         <v>11.879291358187199</v>
       </c>
     </row>
-    <row r="176" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A176" s="4">
         <v>174</v>
       </c>
@@ -15274,7 +15265,7 @@
         <v>11.6775344168566</v>
       </c>
     </row>
-    <row r="177" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A177" s="4">
         <v>175</v>
       </c>
@@ -15356,7 +15347,7 @@
         <v>11.642109123715301</v>
       </c>
     </row>
-    <row r="178" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A178" s="4">
         <v>176</v>
       </c>
@@ -15438,7 +15429,7 @@
         <v>11.498276887877999</v>
       </c>
     </row>
-    <row r="179" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A179" s="4">
         <v>177</v>
       </c>
@@ -15520,7 +15511,7 @@
         <v>11.5180480427939</v>
       </c>
     </row>
-    <row r="180" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A180" s="4">
         <v>178</v>
       </c>
@@ -15602,7 +15593,7 @@
         <v>12.1146615703083</v>
       </c>
     </row>
-    <row r="181" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A181" s="4">
         <v>179</v>
       </c>
@@ -15684,7 +15675,7 @@
         <v>12.2565823130744</v>
       </c>
     </row>
-    <row r="182" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A182" s="4">
         <v>180</v>
       </c>
@@ -15766,7 +15757,7 @@
         <v>12.2678793832705</v>
       </c>
     </row>
-    <row r="183" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A183" s="4">
         <v>181</v>
       </c>
@@ -15848,7 +15839,7 @@
         <v>12.4294502367413</v>
       </c>
     </row>
-    <row r="184" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A184" s="4">
         <v>182</v>
       </c>
@@ -15930,7 +15921,7 @@
         <v>12.361304498200401</v>
       </c>
     </row>
-    <row r="185" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A185" s="4">
         <v>183</v>
       </c>
@@ -16012,7 +16003,7 @@
         <v>11.866143483161499</v>
       </c>
     </row>
-    <row r="186" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A186" s="4">
         <v>184</v>
       </c>
@@ -16094,7 +16085,7 @@
         <v>11.467767805282801</v>
       </c>
     </row>
-    <row r="187" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A187" s="4">
         <v>185</v>
       </c>
@@ -16176,7 +16167,7 @@
         <v>11.445273740109201</v>
       </c>
     </row>
-    <row r="188" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A188" s="4">
         <v>186</v>
       </c>
@@ -16258,7 +16249,7 @@
         <v>11.3991893073767</v>
       </c>
     </row>
-    <row r="189" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A189" s="4">
         <v>187</v>
       </c>
@@ -16340,7 +16331,7 @@
         <v>11.8936194473648</v>
       </c>
     </row>
-    <row r="190" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A190" s="4">
         <v>188</v>
       </c>
@@ -16422,7 +16413,7 @@
         <v>12.7062609107585</v>
       </c>
     </row>
-    <row r="191" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A191" s="4">
         <v>189</v>
       </c>
@@ -16504,7 +16495,7 @@
         <v>13.6572585725811</v>
       </c>
     </row>
-    <row r="192" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A192" s="4">
         <v>190</v>
       </c>
@@ -16586,7 +16577,7 @@
         <v>14.747016123276699</v>
       </c>
     </row>
-    <row r="193" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A193" s="4">
         <v>191</v>
       </c>
@@ -16668,7 +16659,7 @@
         <v>16.282048374839999</v>
       </c>
     </row>
-    <row r="194" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A194" s="4">
         <v>192</v>
       </c>
@@ -16750,7 +16741,7 @@
         <v>17.712003983233199</v>
       </c>
     </row>
-    <row r="195" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A195" s="4">
         <v>193</v>
       </c>
@@ -16832,7 +16823,7 @@
         <v>18.5918000980394</v>
       </c>
     </row>
-    <row r="196" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A196" s="4">
         <v>194</v>
       </c>
@@ -16914,7 +16905,7 @@
         <v>19.498445742313798</v>
       </c>
     </row>
-    <row r="197" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A197" s="4">
         <v>195</v>
       </c>
@@ -16996,7 +16987,7 @@
         <v>20.2589605402109</v>
       </c>
     </row>
-    <row r="198" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A198" s="4">
         <v>196</v>
       </c>
@@ -17078,7 +17069,7 @@
         <v>20.544887992854999</v>
       </c>
     </row>
-    <row r="199" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A199" s="4">
         <v>197</v>
       </c>
@@ -17160,7 +17151,7 @@
         <v>20.932015121038699</v>
       </c>
     </row>
-    <row r="200" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A200" s="4">
         <v>198</v>
       </c>
@@ -17242,7 +17233,7 @@
         <v>21.681003499998699</v>
       </c>
     </row>
-    <row r="201" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A201" s="4">
         <v>199</v>
       </c>
@@ -17324,7 +17315,7 @@
         <v>22.379617101271698</v>
       </c>
     </row>
-    <row r="202" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A202" s="4">
         <v>200</v>
       </c>
@@ -17406,7 +17397,7 @@
         <v>23.488704368278199</v>
       </c>
     </row>
-    <row r="203" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A203" s="4">
         <v>201</v>
       </c>
@@ -17488,7 +17479,7 @@
         <v>23.8833827363759</v>
       </c>
     </row>
-    <row r="204" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A204" s="4">
         <v>202</v>
       </c>
@@ -17570,7 +17561,7 @@
         <v>24.870522999988498</v>
       </c>
     </row>
-    <row r="205" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A205" s="4">
         <v>203</v>
       </c>
@@ -17652,7 +17643,7 @@
         <v>26.040624648346299</v>
       </c>
     </row>
-    <row r="206" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A206" s="4">
         <v>204</v>
       </c>
@@ -17734,7 +17725,7 @@
         <v>27.419787398359698</v>
       </c>
     </row>
-    <row r="207" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A207" s="4">
         <v>205</v>
       </c>
@@ -17816,7 +17807,7 @@
         <v>27.407198372818101</v>
       </c>
     </row>
-    <row r="208" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A208" s="4">
         <v>206</v>
       </c>
@@ -17898,7 +17889,7 @@
         <v>27.260156916497198</v>
       </c>
     </row>
-    <row r="209" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A209" s="4">
         <v>207</v>
       </c>
@@ -17980,7 +17971,7 @@
         <v>27.811560559992301</v>
       </c>
     </row>
-    <row r="210" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A210" s="4">
         <v>208</v>
       </c>
@@ -18062,7 +18053,7 @@
         <v>28.323578228952101</v>
       </c>
     </row>
-    <row r="211" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A211" s="4">
         <v>209</v>
       </c>
@@ -18144,7 +18135,7 @@
         <v>28.810641176833901</v>
       </c>
     </row>
-    <row r="212" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A212" s="4">
         <v>210</v>
       </c>
@@ -18226,7 +18217,7 @@
         <v>29.654156738617399</v>
       </c>
     </row>
-    <row r="213" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A213" s="4">
         <v>211</v>
       </c>
@@ -18308,7 +18299,7 @@
         <v>30.012186955780201</v>
       </c>
     </row>
-    <row r="214" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A214" s="4">
         <v>212</v>
       </c>
@@ -18390,7 +18381,7 @@
         <v>30.6023842791951</v>
       </c>
     </row>
-    <row r="215" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A215" s="4">
         <v>213</v>
       </c>
@@ -18472,7 +18463,7 @@
         <v>31.4350163904464</v>
       </c>
     </row>
-    <row r="216" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A216" s="4">
         <v>214</v>
       </c>
@@ -18554,7 +18545,7 @@
         <v>31.3571049186111</v>
       </c>
     </row>
-    <row r="217" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A217" s="4">
         <v>215</v>
       </c>
@@ -18636,7 +18627,7 @@
         <v>31.7406383790298</v>
       </c>
     </row>
-    <row r="218" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A218" s="4">
         <v>216</v>
       </c>
@@ -18718,7 +18709,7 @@
         <v>31.238266851310399</v>
       </c>
     </row>
-    <row r="219" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A219" s="4">
         <v>217</v>
       </c>
@@ -18800,7 +18791,7 @@
         <v>30.771779004142399</v>
       </c>
     </row>
-    <row r="220" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A220" s="4">
         <v>218</v>
       </c>
@@ -18882,7 +18873,7 @@
         <v>29.168230146264602</v>
       </c>
     </row>
-    <row r="221" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A221" s="4">
         <v>219</v>
       </c>
@@ -18964,7 +18955,7 @@
         <v>27.3320785577477</v>
       </c>
     </row>
-    <row r="222" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A222" s="4">
         <v>220</v>
       </c>
@@ -19046,7 +19037,7 @@
         <v>26.600198382884098</v>
       </c>
     </row>
-    <row r="223" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A223" s="4">
         <v>221</v>
       </c>
@@ -19128,7 +19119,7 @@
         <v>25.899312218927399</v>
       </c>
     </row>
-    <row r="224" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A224" s="4">
         <v>222</v>
       </c>
@@ -19210,7 +19201,7 @@
         <v>25.248489352396099</v>
       </c>
     </row>
-    <row r="225" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A225" s="4">
         <v>223</v>
       </c>
@@ -19292,7 +19283,7 @@
         <v>24.975190286153602</v>
       </c>
     </row>
-    <row r="226" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A226" s="4">
         <v>224</v>
       </c>
@@ -19374,7 +19365,7 @@
         <v>24.797327877659001</v>
       </c>
     </row>
-    <row r="227" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A227" s="4">
         <v>225</v>
       </c>
@@ -19456,7 +19447,7 @@
         <v>24.886786227867599</v>
       </c>
     </row>
-    <row r="228" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A228" s="4">
         <v>226</v>
       </c>
@@ -19538,7 +19529,7 @@
         <v>25.231215737617799</v>
       </c>
     </row>
-    <row r="229" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A229" s="4">
         <v>227</v>
       </c>
@@ -19620,7 +19611,7 @@
         <v>25.743601967571902</v>
       </c>
     </row>
-    <row r="230" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A230" s="4">
         <v>228</v>
       </c>
@@ -19702,7 +19693,7 @@
         <v>26.763867884306698</v>
       </c>
     </row>
-    <row r="231" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A231" s="4">
         <v>229</v>
       </c>
@@ -19784,7 +19775,7 @@
         <v>26.889232646338399</v>
       </c>
     </row>
-    <row r="232" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A232" s="4">
         <v>230</v>
       </c>
@@ -19866,7 +19857,7 @@
         <v>27.378564049755699</v>
       </c>
     </row>
-    <row r="233" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A233" s="4">
         <v>231</v>
       </c>
@@ -19948,7 +19939,7 @@
         <v>26.722578457910199</v>
       </c>
     </row>
-    <row r="234" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A234" s="4">
         <v>232</v>
       </c>
@@ -20030,7 +20021,7 @@
         <v>26.0433872363791</v>
       </c>
     </row>
-    <row r="235" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A235" s="4">
         <v>233</v>
       </c>
@@ -20112,7 +20103,7 @@
         <v>25.432565694878299</v>
       </c>
     </row>
-    <row r="236" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A236" s="4">
         <v>234</v>
       </c>
@@ -20194,7 +20185,7 @@
         <v>24.736998515986201</v>
       </c>
     </row>
-    <row r="237" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A237" s="4">
         <v>235</v>
       </c>
@@ -20276,7 +20267,7 @@
         <v>24.240650205704</v>
       </c>
     </row>
-    <row r="238" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A238" s="4">
         <v>236</v>
       </c>
@@ -20358,7 +20349,7 @@
         <v>23.9990279894261</v>
       </c>
     </row>
-    <row r="239" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A239" s="4">
         <v>237</v>
       </c>
@@ -20440,7 +20431,7 @@
         <v>24.503548672513901</v>
       </c>
     </row>
-    <row r="240" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A240" s="4">
         <v>238</v>
       </c>
@@ -20522,7 +20513,7 @@
         <v>25.134537340839</v>
       </c>
     </row>
-    <row r="241" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A241" s="4">
         <v>239</v>
       </c>
@@ -20604,7 +20595,7 @@
         <v>25.865718685452102</v>
       </c>
     </row>
-    <row r="242" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A242" s="4">
         <v>240</v>
       </c>
@@ -20686,7 +20677,7 @@
         <v>26.2121296786252</v>
       </c>
     </row>
-    <row r="243" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A243" s="4">
         <v>241</v>
       </c>
@@ -20768,7 +20759,7 @@
         <v>27.306221620894199</v>
       </c>
     </row>
-    <row r="244" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A244" s="4">
         <v>242</v>
       </c>
@@ -20850,7 +20841,7 @@
         <v>28.7289945657628</v>
       </c>
     </row>
-    <row r="245" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A245" s="4">
         <v>243</v>
       </c>
@@ -20932,7 +20923,7 @@
         <v>30.081878929691499</v>
       </c>
     </row>
-    <row r="246" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A246" s="4">
         <v>244</v>
       </c>
@@ -21014,7 +21005,7 @@
         <v>29.953416350638701</v>
       </c>
     </row>
-    <row r="247" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A247" s="4">
         <v>245</v>
       </c>
@@ -21096,7 +21087,7 @@
         <v>30.122000749080701</v>
       </c>
     </row>
-    <row r="248" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A248" s="4">
         <v>246</v>
       </c>
@@ -21178,7 +21169,7 @@
         <v>29.764326961141901</v>
       </c>
     </row>
-    <row r="249" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A249" s="4">
         <v>247</v>
       </c>
@@ -21260,7 +21251,7 @@
         <v>29.316410221164901</v>
       </c>
     </row>
-    <row r="250" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A250" s="4">
         <v>248</v>
       </c>
@@ -21308,7 +21299,7 @@
         <f>100*testdata[[#This Row],[-DM14]]/testdata[[#This Row],[TR14]]</f>
         <v>18.247083794191962</v>
       </c>
-      <c r="N250" s="6">
+      <c r="N250" s="11">
         <f>100*ABS(testdata[[#This Row],[+DI14]]-testdata[[#This Row],[-DI14]])/(testdata[[#This Row],[+DI14]]+testdata[[#This Row],[-DI14]])</f>
         <v>27.825450922906132</v>
       </c>
@@ -21342,7 +21333,7 @@
         <v>29.125166308423101</v>
       </c>
     </row>
-    <row r="251" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A251" s="4">
         <v>249</v>
       </c>
@@ -21424,7 +21415,7 @@
         <v>29.2164317967156</v>
       </c>
     </row>
-    <row r="252" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A252" s="4">
         <v>250</v>
       </c>
@@ -21506,7 +21497,7 @@
         <v>29.079359374489599</v>
       </c>
     </row>
-    <row r="253" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A253" s="4">
         <v>251</v>
       </c>
@@ -21588,7 +21579,7 @@
         <v>29.1949732270187</v>
       </c>
     </row>
-    <row r="254" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A254" s="4">
         <v>252</v>
       </c>
@@ -21670,7 +21661,7 @@
         <v>29.833025880740301</v>
       </c>
     </row>
-    <row r="255" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A255" s="4">
         <v>253</v>
       </c>
@@ -21752,7 +21743,7 @@
         <v>30.321430073304999</v>
       </c>
     </row>
-    <row r="256" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A256" s="4">
         <v>254</v>
       </c>
@@ -21834,7 +21825,7 @@
         <v>31.241288391566101</v>
       </c>
     </row>
-    <row r="257" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A257" s="4">
         <v>255</v>
       </c>
@@ -21916,7 +21907,7 @@
         <v>32.442144175962397</v>
       </c>
     </row>
-    <row r="258" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A258" s="4">
         <v>256</v>
       </c>
@@ -21998,7 +21989,7 @@
         <v>33.380723590489403</v>
       </c>
     </row>
-    <row r="259" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A259" s="4">
         <v>257</v>
       </c>
@@ -22080,7 +22071,7 @@
         <v>33.576693497222898</v>
       </c>
     </row>
-    <row r="260" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A260" s="4">
         <v>258</v>
       </c>
@@ -22162,7 +22153,7 @@
         <v>34.039171782289998</v>
       </c>
     </row>
-    <row r="261" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A261" s="4">
         <v>259</v>
       </c>
@@ -22244,7 +22235,7 @@
         <v>34.5633153964095</v>
       </c>
     </row>
-    <row r="262" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A262" s="4">
         <v>260</v>
       </c>
@@ -22326,7 +22317,7 @@
         <v>35.243272783614103</v>
       </c>
     </row>
-    <row r="263" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A263" s="4">
         <v>261</v>
       </c>
@@ -22408,7 +22399,7 @@
         <v>35.9498050617091</v>
       </c>
     </row>
-    <row r="264" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A264" s="4">
         <v>262</v>
       </c>
@@ -22490,7 +22481,7 @@
         <v>36.655447226794401</v>
       </c>
     </row>
-    <row r="265" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A265" s="4">
         <v>263</v>
       </c>
@@ -22572,7 +22563,7 @@
         <v>36.978448067860199</v>
       </c>
     </row>
-    <row r="266" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A266" s="4">
         <v>264</v>
       </c>
@@ -22654,7 +22645,7 @@
         <v>37.571222731222598</v>
       </c>
     </row>
-    <row r="267" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A267" s="4">
         <v>265</v>
       </c>
@@ -22736,7 +22727,7 @@
         <v>38.683797841457</v>
       </c>
     </row>
-    <row r="268" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A268" s="4">
         <v>266</v>
       </c>
@@ -22818,7 +22809,7 @@
         <v>40.108469578976297</v>
       </c>
     </row>
-    <row r="269" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A269" s="4">
         <v>267</v>
       </c>
@@ -22900,7 +22891,7 @@
         <v>41.669773300721502</v>
       </c>
     </row>
-    <row r="270" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A270" s="4">
         <v>268</v>
       </c>
@@ -22982,7 +22973,7 @@
         <v>43.355401407904203</v>
       </c>
     </row>
-    <row r="271" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A271" s="4">
         <v>269</v>
       </c>
@@ -23064,7 +23055,7 @@
         <v>45.0853097599989</v>
       </c>
     </row>
-    <row r="272" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A272" s="4">
         <v>270</v>
       </c>
@@ -23146,7 +23137,7 @@
         <v>44.8302113134135</v>
       </c>
     </row>
-    <row r="273" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A273" s="4">
         <v>271</v>
       </c>
@@ -23228,7 +23219,7 @@
         <v>44.682997203934796</v>
       </c>
     </row>
-    <row r="274" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A274" s="4">
         <v>272</v>
       </c>
@@ -23310,7 +23301,7 @@
         <v>44.800202646040198</v>
       </c>
     </row>
-    <row r="275" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A275" s="4">
         <v>273</v>
       </c>
@@ -23392,7 +23383,7 @@
         <v>43.949283404165698</v>
       </c>
     </row>
-    <row r="276" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A276" s="4">
         <v>274</v>
       </c>
@@ -23474,7 +23465,7 @@
         <v>44.595460482788901</v>
       </c>
     </row>
-    <row r="277" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A277" s="4">
         <v>275</v>
       </c>
@@ -23556,7 +23547,7 @@
         <v>45.489532518218297</v>
       </c>
     </row>
-    <row r="278" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A278" s="4">
         <v>276</v>
       </c>
@@ -23638,7 +23629,7 @@
         <v>45.917445996110096</v>
       </c>
     </row>
-    <row r="279" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A279" s="4">
         <v>277</v>
       </c>
@@ -23720,7 +23711,7 @@
         <v>47.073628957847298</v>
       </c>
     </row>
-    <row r="280" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A280" s="4">
         <v>278</v>
       </c>
@@ -23802,7 +23793,7 @@
         <v>48.402261377820203</v>
       </c>
     </row>
-    <row r="281" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A281" s="4">
         <v>279</v>
       </c>
@@ -23884,7 +23875,7 @@
         <v>49.253150487665899</v>
       </c>
     </row>
-    <row r="282" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A282" s="4">
         <v>280</v>
       </c>
@@ -23966,7 +23957,7 @@
         <v>50.043261803951097</v>
       </c>
     </row>
-    <row r="283" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A283" s="4">
         <v>281</v>
       </c>
@@ -24048,7 +24039,7 @@
         <v>50.482810002419299</v>
       </c>
     </row>
-    <row r="284" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A284" s="4">
         <v>282</v>
       </c>
@@ -24130,7 +24121,7 @@
         <v>50.524515847224599</v>
       </c>
     </row>
-    <row r="285" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A285" s="4">
         <v>283</v>
       </c>
@@ -24212,7 +24203,7 @@
         <v>48.9727311126397</v>
       </c>
     </row>
-    <row r="286" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A286" s="4">
         <v>284</v>
       </c>
@@ -24294,7 +24285,7 @@
         <v>47.489243388807999</v>
       </c>
     </row>
-    <row r="287" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A287" s="4">
         <v>285</v>
       </c>
@@ -24376,7 +24367,7 @@
         <v>45.988055235207099</v>
       </c>
     </row>
-    <row r="288" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A288" s="4">
         <v>286</v>
       </c>
@@ -24458,7 +24449,7 @@
         <v>43.458459724148398</v>
       </c>
     </row>
-    <row r="289" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A289" s="4">
         <v>287</v>
       </c>
@@ -24540,7 +24531,7 @@
         <v>42.336710251636497</v>
       </c>
     </row>
-    <row r="290" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A290" s="4">
         <v>288</v>
       </c>
@@ -24622,7 +24613,7 @@
         <v>41.204624480284501</v>
       </c>
     </row>
-    <row r="291" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A291" s="4">
         <v>289</v>
       </c>
@@ -24704,7 +24695,7 @@
         <v>39.703261507314402</v>
       </c>
     </row>
-    <row r="292" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A292" s="4">
         <v>290</v>
       </c>
@@ -24786,7 +24777,7 @@
         <v>39.186372254460899</v>
       </c>
     </row>
-    <row r="293" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A293" s="4">
         <v>291</v>
       </c>
@@ -24868,7 +24859,7 @@
         <v>39.364514982524398</v>
       </c>
     </row>
-    <row r="294" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A294" s="4">
         <v>292</v>
       </c>
@@ -24950,7 +24941,7 @@
         <v>39.162926652029299</v>
       </c>
     </row>
-    <row r="295" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A295" s="4">
         <v>293</v>
       </c>
@@ -25032,7 +25023,7 @@
         <v>38.5659328083131</v>
       </c>
     </row>
-    <row r="296" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A296" s="4">
         <v>294</v>
       </c>
@@ -25114,7 +25105,7 @@
         <v>37.502797409335997</v>
       </c>
     </row>
-    <row r="297" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A297" s="4">
         <v>295</v>
       </c>
@@ -25196,7 +25187,7 @@
         <v>36.244865030022403</v>
       </c>
     </row>
-    <row r="298" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A298" s="4">
         <v>296</v>
       </c>
@@ -25278,7 +25269,7 @@
         <v>34.674984555811697</v>
       </c>
     </row>
-    <row r="299" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A299" s="4">
         <v>297</v>
       </c>
@@ -25360,7 +25351,7 @@
         <v>33.072077162676301</v>
       </c>
     </row>
-    <row r="300" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A300" s="4">
         <v>298</v>
       </c>
@@ -25442,7 +25433,7 @@
         <v>31.572873004156001</v>
       </c>
     </row>
-    <row r="301" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A301" s="4">
         <v>299</v>
       </c>
@@ -25524,7 +25515,7 @@
         <v>29.9561712714073</v>
       </c>
     </row>
-    <row r="302" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A302" s="4">
         <v>300</v>
       </c>
@@ -25606,7 +25597,7 @@
         <v>28.400852893868699</v>
       </c>
     </row>
-    <row r="303" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A303" s="4">
         <v>301</v>
       </c>
@@ -25688,7 +25679,7 @@
         <v>26.600677803712301</v>
       </c>
     </row>
-    <row r="304" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A304" s="4">
         <v>302</v>
       </c>
@@ -25770,7 +25761,7 @@
         <v>24.9290866485671</v>
       </c>
     </row>
-    <row r="305" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A305" s="4">
         <v>303</v>
       </c>
@@ -25852,7 +25843,7 @@
         <v>24.330164002215401</v>
       </c>
     </row>
-    <row r="306" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A306" s="4">
         <v>304</v>
       </c>
@@ -25934,7 +25925,7 @@
         <v>24.249288733771099</v>
       </c>
     </row>
-    <row r="307" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A307" s="4">
         <v>305</v>
       </c>
@@ -26016,7 +26007,7 @@
         <v>24.012982288271299</v>
       </c>
     </row>
-    <row r="308" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A308" s="4">
         <v>306</v>
       </c>
@@ -26098,7 +26089,7 @@
         <v>24.021074651591999</v>
       </c>
     </row>
-    <row r="309" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A309" s="4">
         <v>307</v>
       </c>
@@ -26180,7 +26171,7 @@
         <v>24.3361205913288</v>
       </c>
     </row>
-    <row r="310" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A310" s="4">
         <v>308</v>
       </c>
@@ -26262,7 +26253,7 @@
         <v>24.6609309569155</v>
       </c>
     </row>
-    <row r="311" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A311" s="4">
         <v>309</v>
       </c>
@@ -26344,7 +26335,7 @@
         <v>24.609799024355802</v>
       </c>
     </row>
-    <row r="312" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A312" s="4">
         <v>310</v>
       </c>
@@ -26426,7 +26417,7 @@
         <v>24.299107490012901</v>
       </c>
     </row>
-    <row r="313" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A313" s="4">
         <v>311</v>
       </c>
@@ -26508,7 +26499,7 @@
         <v>23.708973109991799</v>
       </c>
     </row>
-    <row r="314" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A314" s="4">
         <v>312</v>
       </c>
@@ -26590,7 +26581,7 @@
         <v>23.320559083278098</v>
       </c>
     </row>
-    <row r="315" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A315" s="4">
         <v>313</v>
       </c>
@@ -26672,7 +26663,7 @@
         <v>23.114949305379099</v>
       </c>
     </row>
-    <row r="316" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A316" s="4">
         <v>314</v>
       </c>
@@ -26754,7 +26745,7 @@
         <v>22.4902681345764</v>
       </c>
     </row>
-    <row r="317" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A317" s="4">
         <v>315</v>
       </c>
@@ -26836,7 +26827,7 @@
         <v>21.5965931053479</v>
       </c>
     </row>
-    <row r="318" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A318" s="4">
         <v>316</v>
       </c>
@@ -26918,7 +26909,7 @@
         <v>21.920946856281098</v>
       </c>
     </row>
-    <row r="319" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A319" s="4">
         <v>317</v>
       </c>
@@ -27000,7 +26991,7 @@
         <v>22.2221324821477</v>
       </c>
     </row>
-    <row r="320" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A320" s="4">
         <v>318</v>
       </c>
@@ -27082,7 +27073,7 @@
         <v>22.075075981773001</v>
       </c>
     </row>
-    <row r="321" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A321" s="4">
         <v>319</v>
       </c>
@@ -27164,7 +27155,7 @@
         <v>22.5758479738234</v>
       </c>
     </row>
-    <row r="322" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A322" s="4">
         <v>320</v>
       </c>
@@ -27246,7 +27237,7 @@
         <v>23.204105080850901</v>
       </c>
     </row>
-    <row r="323" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A323" s="4">
         <v>321</v>
       </c>
@@ -27328,7 +27319,7 @@
         <v>23.831982200405601</v>
       </c>
     </row>
-    <row r="324" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A324" s="4">
         <v>322</v>
       </c>
@@ -27410,7 +27401,7 @@
         <v>24.100669583639199</v>
       </c>
     </row>
-    <row r="325" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A325" s="4">
         <v>323</v>
       </c>
@@ -27492,7 +27483,7 @@
         <v>23.957310799270498</v>
       </c>
     </row>
-    <row r="326" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A326" s="4">
         <v>324</v>
       </c>
@@ -27574,7 +27565,7 @@
         <v>23.347236408235101</v>
       </c>
     </row>
-    <row r="327" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A327" s="4">
         <v>325</v>
       </c>
@@ -27656,7 +27647,7 @@
         <v>23.465210872016701</v>
       </c>
     </row>
-    <row r="328" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A328" s="4">
         <v>326</v>
       </c>
@@ -27738,7 +27729,7 @@
         <v>23.819705472483701</v>
       </c>
     </row>
-    <row r="329" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A329" s="4">
         <v>327</v>
       </c>
@@ -27820,7 +27811,7 @@
         <v>23.716015492394899</v>
       </c>
     </row>
-    <row r="330" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A330" s="4">
         <v>328</v>
       </c>
@@ -27902,7 +27893,7 @@
         <v>23.7268905067628</v>
       </c>
     </row>
-    <row r="331" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A331" s="4">
         <v>329</v>
       </c>
@@ -27984,7 +27975,7 @@
         <v>24.308211406051001</v>
       </c>
     </row>
-    <row r="332" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A332" s="4">
         <v>330</v>
       </c>
@@ -28066,7 +28057,7 @@
         <v>24.296009563747699</v>
       </c>
     </row>
-    <row r="333" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A333" s="4">
         <v>331</v>
       </c>
@@ -28148,7 +28139,7 @@
         <v>24.0975316290112</v>
       </c>
     </row>
-    <row r="334" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A334" s="4">
         <v>332</v>
       </c>
@@ -28230,7 +28221,7 @@
         <v>24.040589746413101</v>
       </c>
     </row>
-    <row r="335" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A335" s="4">
         <v>333</v>
       </c>
@@ -28312,7 +28303,7 @@
         <v>24.040297779885101</v>
       </c>
     </row>
-    <row r="336" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A336" s="4">
         <v>334</v>
       </c>
@@ -28394,7 +28385,7 @@
         <v>24.0358557453396</v>
       </c>
     </row>
-    <row r="337" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A337" s="4">
         <v>335</v>
       </c>
@@ -28476,7 +28467,7 @@
         <v>24.3059452059323</v>
       </c>
     </row>
-    <row r="338" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A338" s="4">
         <v>336</v>
       </c>
@@ -28558,7 +28549,7 @@
         <v>23.5333877332789</v>
       </c>
     </row>
-    <row r="339" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A339" s="4">
         <v>337</v>
       </c>
@@ -28640,7 +28631,7 @@
         <v>22.5567838939</v>
       </c>
     </row>
-    <row r="340" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A340" s="4">
         <v>338</v>
       </c>
@@ -28722,7 +28713,7 @@
         <v>22.037988007839701</v>
       </c>
     </row>
-    <row r="341" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A341" s="4">
         <v>339</v>
       </c>
@@ -28804,7 +28795,7 @@
         <v>21.400084393895899</v>
       </c>
     </row>
-    <row r="342" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A342" s="4">
         <v>340</v>
       </c>
@@ -28886,7 +28877,7 @@
         <v>20.774055296181899</v>
       </c>
     </row>
-    <row r="343" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A343" s="4">
         <v>341</v>
       </c>
@@ -28968,7 +28959,7 @@
         <v>20.713454193698698</v>
       </c>
     </row>
-    <row r="344" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A344" s="4">
         <v>342</v>
       </c>
@@ -29050,7 +29041,7 @@
         <v>20.820641487708102</v>
       </c>
     </row>
-    <row r="345" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A345" s="4">
         <v>343</v>
       </c>
@@ -29132,7 +29123,7 @@
         <v>20.007212094078799</v>
       </c>
     </row>
-    <row r="346" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A346" s="4">
         <v>344</v>
       </c>
@@ -29214,7 +29205,7 @@
         <v>19.400862031148701</v>
       </c>
     </row>
-    <row r="347" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A347" s="4">
         <v>345</v>
       </c>
@@ -29296,7 +29287,7 @@
         <v>19.033849901852602</v>
       </c>
     </row>
-    <row r="348" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A348" s="4">
         <v>346</v>
       </c>
@@ -29378,7 +29369,7 @@
         <v>18.916167065472699</v>
       </c>
     </row>
-    <row r="349" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A349" s="4">
         <v>347</v>
       </c>
@@ -29460,7 +29451,7 @@
         <v>18.9864164410826</v>
       </c>
     </row>
-    <row r="350" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A350" s="4">
         <v>348</v>
       </c>
@@ -29542,7 +29533,7 @@
         <v>19.4721973298854</v>
       </c>
     </row>
-    <row r="351" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A351" s="4">
         <v>349</v>
       </c>
@@ -29624,7 +29615,7 @@
         <v>19.065660266944601</v>
       </c>
     </row>
-    <row r="352" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A352" s="4">
         <v>350</v>
       </c>
@@ -29706,7 +29697,7 @@
         <v>18.450557253607801</v>
       </c>
     </row>
-    <row r="353" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A353" s="4">
         <v>351</v>
       </c>
@@ -29788,7 +29779,7 @@
         <v>17.993188939884899</v>
       </c>
     </row>
-    <row r="354" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A354" s="4">
         <v>352</v>
       </c>
@@ -29870,7 +29861,7 @@
         <v>17.370528133367301</v>
       </c>
     </row>
-    <row r="355" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A355" s="4">
         <v>353</v>
       </c>
@@ -29952,7 +29943,7 @@
         <v>16.361103887229799</v>
       </c>
     </row>
-    <row r="356" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A356" s="4">
         <v>354</v>
       </c>
@@ -30034,7 +30025,7 @@
         <v>15.552843087417999</v>
       </c>
     </row>
-    <row r="357" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A357" s="4">
         <v>355</v>
       </c>
@@ -30116,7 +30107,7 @@
         <v>14.9670865577054</v>
       </c>
     </row>
-    <row r="358" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A358" s="4">
         <v>356</v>
       </c>
@@ -30198,7 +30189,7 @@
         <v>14.2776973816188</v>
       </c>
     </row>
-    <row r="359" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A359" s="4">
         <v>357</v>
       </c>
@@ -30280,7 +30271,7 @@
         <v>13.8608899240038</v>
       </c>
     </row>
-    <row r="360" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A360" s="4">
         <v>358</v>
       </c>
@@ -30362,7 +30353,7 @@
         <v>13.8678426711318</v>
       </c>
     </row>
-    <row r="361" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A361" s="4">
         <v>359</v>
       </c>
@@ -30444,7 +30435,7 @@
         <v>13.9525434693052</v>
       </c>
     </row>
-    <row r="362" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A362" s="4">
         <v>360</v>
       </c>
@@ -30526,7 +30517,7 @@
         <v>14.3228300719055</v>
       </c>
     </row>
-    <row r="363" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A363" s="4">
         <v>361</v>
       </c>
@@ -30608,7 +30599,7 @@
         <v>14.884309733596799</v>
       </c>
     </row>
-    <row r="364" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A364" s="4">
         <v>362</v>
       </c>
@@ -30690,7 +30681,7 @@
         <v>15.1235247980179</v>
       </c>
     </row>
-    <row r="365" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A365" s="4">
         <v>363</v>
       </c>
@@ -30772,7 +30763,7 @@
         <v>15.190511916975399</v>
       </c>
     </row>
-    <row r="366" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A366" s="4">
         <v>364</v>
       </c>
@@ -30854,7 +30845,7 @@
         <v>15.2527142417217</v>
       </c>
     </row>
-    <row r="367" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A367" s="4">
         <v>365</v>
       </c>
@@ -30936,7 +30927,7 @@
         <v>15.064245297757999</v>
       </c>
     </row>
-    <row r="368" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A368" s="4">
         <v>366</v>
       </c>
@@ -31018,7 +31009,7 @@
         <v>14.4087144661494</v>
       </c>
     </row>
-    <row r="369" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A369" s="4">
         <v>367</v>
       </c>
@@ -31100,7 +31091,7 @@
         <v>13.5452486298121</v>
       </c>
     </row>
-    <row r="370" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A370" s="4">
         <v>368</v>
       </c>
@@ -31182,7 +31173,7 @@
         <v>12.9272276871381</v>
       </c>
     </row>
-    <row r="371" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A371" s="4">
         <v>369</v>
       </c>
@@ -31264,7 +31255,7 @@
         <v>12.6547212717257</v>
       </c>
     </row>
-    <row r="372" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A372" s="4">
         <v>370</v>
       </c>
@@ -31346,7 +31337,7 @@
         <v>12.4603744291437</v>
       </c>
     </row>
-    <row r="373" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A373" s="4">
         <v>371</v>
       </c>
@@ -31428,7 +31419,7 @@
         <v>13.563590916138001</v>
       </c>
     </row>
-    <row r="374" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A374" s="4">
         <v>372</v>
       </c>
@@ -31510,7 +31501,7 @@
         <v>14.7019891631258</v>
       </c>
     </row>
-    <row r="375" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A375" s="4">
         <v>373</v>
       </c>
@@ -31592,7 +31583,7 @@
         <v>15.972210649169</v>
       </c>
     </row>
-    <row r="376" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A376" s="4">
         <v>374</v>
       </c>
@@ -31674,7 +31665,7 @@
         <v>17.4146380538457</v>
       </c>
     </row>
-    <row r="377" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A377" s="4">
         <v>375</v>
       </c>
@@ -31756,7 +31747,7 @@
         <v>18.168954250697599</v>
       </c>
     </row>
-    <row r="378" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A378" s="4">
         <v>376</v>
       </c>
@@ -31838,7 +31829,7 @@
         <v>19.023318463398201</v>
       </c>
     </row>
-    <row r="379" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A379" s="4">
         <v>377</v>
       </c>
@@ -31920,7 +31911,7 @@
         <v>19.565028793365201</v>
       </c>
     </row>
-    <row r="380" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A380" s="4">
         <v>378</v>
       </c>
@@ -32002,7 +31993,7 @@
         <v>19.562903121324101</v>
       </c>
     </row>
-    <row r="381" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A381" s="4">
         <v>379</v>
       </c>
@@ -32084,7 +32075,7 @@
         <v>18.794050732586101</v>
       </c>
     </row>
-    <row r="382" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A382" s="4">
         <v>380</v>
       </c>
@@ -32166,7 +32157,7 @@
         <v>17.636341940310299</v>
       </c>
     </row>
-    <row r="383" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A383" s="4">
         <v>381</v>
       </c>
@@ -32248,7 +32239,7 @@
         <v>16.8959692304635</v>
       </c>
     </row>
-    <row r="384" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A384" s="4">
         <v>382</v>
       </c>
@@ -32330,7 +32321,7 @@
         <v>15.9743349349905</v>
       </c>
     </row>
-    <row r="385" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A385" s="4">
         <v>383</v>
       </c>
@@ -32412,7 +32403,7 @@
         <v>15.378211183727</v>
       </c>
     </row>
-    <row r="386" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A386" s="4">
         <v>384</v>
       </c>
@@ -32494,7 +32485,7 @@
         <v>15.8727196009918</v>
       </c>
     </row>
-    <row r="387" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A387" s="4">
         <v>385</v>
       </c>
@@ -32576,7 +32567,7 @@
         <v>16.331905988451901</v>
       </c>
     </row>
-    <row r="388" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A388" s="4">
         <v>386</v>
       </c>
@@ -32658,7 +32649,7 @@
         <v>17.1822329095613</v>
       </c>
     </row>
-    <row r="389" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A389" s="4">
         <v>387</v>
       </c>
@@ -32740,7 +32731,7 @@
         <v>18.110362038823698</v>
       </c>
     </row>
-    <row r="390" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A390" s="4">
         <v>388</v>
       </c>
@@ -32822,7 +32813,7 @@
         <v>18.2596895435288</v>
       </c>
     </row>
-    <row r="391" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A391" s="4">
         <v>389</v>
       </c>
@@ -32904,7 +32895,7 @@
         <v>18.666597694851198</v>
       </c>
     </row>
-    <row r="392" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A392" s="4">
         <v>390</v>
       </c>
@@ -32986,7 +32977,7 @@
         <v>18.6654025041172</v>
       </c>
     </row>
-    <row r="393" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A393" s="4">
         <v>391</v>
       </c>
@@ -33068,7 +33059,7 @@
         <v>19.074902798161101</v>
       </c>
     </row>
-    <row r="394" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A394" s="4">
         <v>392</v>
       </c>
@@ -33150,7 +33141,7 @@
         <v>19.123796163093498</v>
       </c>
     </row>
-    <row r="395" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A395" s="4">
         <v>393</v>
       </c>
@@ -33232,7 +33223,7 @@
         <v>19.009303941781699</v>
       </c>
     </row>
-    <row r="396" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A396" s="4">
         <v>394</v>
       </c>
@@ -33314,7 +33305,7 @@
         <v>18.307842361126099</v>
       </c>
     </row>
-    <row r="397" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A397" s="4">
         <v>395</v>
       </c>
@@ -33396,7 +33387,7 @@
         <v>17.0879358103426</v>
       </c>
     </row>
-    <row r="398" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A398" s="4">
         <v>396</v>
       </c>
@@ -33478,7 +33469,7 @@
         <v>16.290524284807301</v>
       </c>
     </row>
-    <row r="399" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A399" s="4">
         <v>397</v>
       </c>
@@ -33560,7 +33551,7 @@
         <v>15.575556265207601</v>
       </c>
     </row>
-    <row r="400" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A400" s="4">
         <v>398</v>
       </c>
@@ -33642,7 +33633,7 @@
         <v>14.974989311149301</v>
       </c>
     </row>
-    <row r="401" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A401" s="4">
         <v>399</v>
       </c>
@@ -33724,7 +33715,7 @@
         <v>14.592319179051501</v>
       </c>
     </row>
-    <row r="402" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A402" s="4">
         <v>400</v>
       </c>
@@ -33806,7 +33797,7 @@
         <v>14.6044250109464</v>
       </c>
     </row>
-    <row r="403" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A403" s="4">
         <v>401</v>
       </c>
@@ -33888,7 +33879,7 @@
         <v>14.670969027999099</v>
       </c>
     </row>
-    <row r="404" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A404" s="4">
         <v>402</v>
       </c>
@@ -33970,7 +33961,7 @@
         <v>14.641936624316999</v>
       </c>
     </row>
-    <row r="405" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A405" s="4">
         <v>403</v>
       </c>
@@ -34052,7 +34043,7 @@
         <v>14.501903250587301</v>
       </c>
     </row>
-    <row r="406" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A406" s="4">
         <v>404</v>
       </c>
@@ -34134,7 +34125,7 @@
         <v>14.408782776300701</v>
       </c>
     </row>
-    <row r="407" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A407" s="4">
         <v>405</v>
       </c>
@@ -34216,7 +34207,7 @@
         <v>14.787537026659299</v>
       </c>
     </row>
-    <row r="408" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A408" s="4">
         <v>406</v>
       </c>
@@ -34298,7 +34289,7 @@
         <v>15.136210145418</v>
       </c>
     </row>
-    <row r="409" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A409" s="4">
         <v>407</v>
       </c>
@@ -34380,7 +34371,7 @@
         <v>15.197387871054801</v>
       </c>
     </row>
-    <row r="410" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A410" s="4">
         <v>408</v>
       </c>
@@ -34462,7 +34453,7 @@
         <v>14.3193647860939</v>
       </c>
     </row>
-    <row r="411" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A411" s="4">
         <v>409</v>
       </c>
@@ -34544,7 +34535,7 @@
         <v>13.455772188056899</v>
       </c>
     </row>
-    <row r="412" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A412" s="4">
         <v>410</v>
       </c>
@@ -34626,7 +34617,7 @@
         <v>12.6872116218054</v>
       </c>
     </row>
-    <row r="413" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A413" s="4">
         <v>411</v>
       </c>
@@ -34708,7 +34699,7 @@
         <v>12.3476066811418</v>
       </c>
     </row>
-    <row r="414" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A414" s="4">
         <v>412</v>
       </c>
@@ -34790,7 +34781,7 @@
         <v>11.958458425863901</v>
       </c>
     </row>
-    <row r="415" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A415" s="4">
         <v>413</v>
       </c>
@@ -34872,7 +34863,7 @@
         <v>11.9543942276407</v>
       </c>
     </row>
-    <row r="416" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A416" s="4">
         <v>414</v>
       </c>
@@ -34954,7 +34945,7 @@
         <v>12.346677481393</v>
       </c>
     </row>
-    <row r="417" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A417" s="4">
         <v>415</v>
       </c>
@@ -35036,7 +35027,7 @@
         <v>13.0859098694095</v>
       </c>
     </row>
-    <row r="418" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A418" s="4">
         <v>416</v>
       </c>
@@ -35118,7 +35109,7 @@
         <v>13.880547133235901</v>
       </c>
     </row>
-    <row r="419" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A419" s="4">
         <v>417</v>
       </c>
@@ -35200,7 +35191,7 @@
         <v>14.4148382275316</v>
       </c>
     </row>
-    <row r="420" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A420" s="4">
         <v>418</v>
       </c>
@@ -35282,7 +35273,7 @@
         <v>14.957807606987</v>
       </c>
     </row>
-    <row r="421" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A421" s="4">
         <v>419</v>
       </c>
@@ -35364,7 +35355,7 @@
         <v>15.3296561037263</v>
       </c>
     </row>
-    <row r="422" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A422" s="4">
         <v>420</v>
       </c>
@@ -35446,7 +35437,7 @@
         <v>15.968613297333301</v>
       </c>
     </row>
-    <row r="423" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A423" s="4">
         <v>421</v>
       </c>
@@ -35528,7 +35519,7 @@
         <v>15.587223497216399</v>
       </c>
     </row>
-    <row r="424" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A424" s="4">
         <v>422</v>
       </c>
@@ -35610,7 +35601,7 @@
         <v>14.807751837768199</v>
       </c>
     </row>
-    <row r="425" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A425" s="4">
         <v>423</v>
       </c>
@@ -35692,7 +35683,7 @@
         <v>14.0858205828425</v>
       </c>
     </row>
-    <row r="426" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A426" s="4">
         <v>424</v>
       </c>
@@ -35774,7 +35765,7 @@
         <v>13.8267905444765</v>
       </c>
     </row>
-    <row r="427" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A427" s="4">
         <v>425</v>
       </c>
@@ -35856,7 +35847,7 @@
         <v>13.239849190144</v>
       </c>
     </row>
-    <row r="428" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A428" s="4">
         <v>426</v>
       </c>
@@ -35938,7 +35929,7 @@
         <v>12.8184044512486</v>
       </c>
     </row>
-    <row r="429" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A429" s="4">
         <v>427</v>
       </c>
@@ -36020,7 +36011,7 @@
         <v>12.9848088164429</v>
       </c>
     </row>
-    <row r="430" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A430" s="4">
         <v>428</v>
       </c>
@@ -36102,7 +36093,7 @@
         <v>13.6733974281626</v>
       </c>
     </row>
-    <row r="431" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A431" s="4">
         <v>429</v>
       </c>
@@ -36184,7 +36175,7 @@
         <v>14.0396838581923</v>
       </c>
     </row>
-    <row r="432" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A432" s="4">
         <v>430</v>
       </c>
@@ -36266,7 +36257,7 @@
         <v>14.830533018637199</v>
       </c>
     </row>
-    <row r="433" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A433" s="4">
         <v>431</v>
       </c>
@@ -36348,7 +36339,7 @@
         <v>15.504727933627199</v>
       </c>
     </row>
-    <row r="434" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A434" s="4">
         <v>432</v>
       </c>
@@ -36430,7 +36421,7 @@
         <v>16.6004438243355</v>
       </c>
     </row>
-    <row r="435" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A435" s="4">
         <v>433</v>
       </c>
@@ -36512,7 +36503,7 @@
         <v>17.520967675199099</v>
       </c>
     </row>
-    <row r="436" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A436" s="4">
         <v>434</v>
       </c>
@@ -36594,7 +36585,7 @@
         <v>17.5201980007906</v>
       </c>
     </row>
-    <row r="437" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A437" s="4">
         <v>435</v>
       </c>
@@ -36676,7 +36667,7 @@
         <v>17.258230265366201</v>
       </c>
     </row>
-    <row r="438" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A438" s="4">
         <v>436</v>
       </c>
@@ -36758,7 +36749,7 @@
         <v>16.526766103900702</v>
       </c>
     </row>
-    <row r="439" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A439" s="4">
         <v>437</v>
       </c>
@@ -36840,7 +36831,7 @@
         <v>15.948157559890999</v>
       </c>
     </row>
-    <row r="440" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A440" s="4">
         <v>438</v>
       </c>
@@ -36922,7 +36913,7 @@
         <v>15.0443602217851</v>
       </c>
     </row>
-    <row r="441" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A441" s="4">
         <v>439</v>
       </c>
@@ -37004,7 +36995,7 @@
         <v>14.787644812962601</v>
       </c>
     </row>
-    <row r="442" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A442" s="4">
         <v>440</v>
       </c>
@@ -37086,7 +37077,7 @@
         <v>14.929267156716</v>
       </c>
     </row>
-    <row r="443" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A443" s="4">
         <v>441</v>
       </c>
@@ -37168,7 +37159,7 @@
         <v>15.363294955236601</v>
       </c>
     </row>
-    <row r="444" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A444" s="4">
         <v>442</v>
       </c>
@@ -37250,7 +37241,7 @@
         <v>14.755581750279401</v>
       </c>
     </row>
-    <row r="445" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A445" s="4">
         <v>443</v>
       </c>
@@ -37332,7 +37323,7 @@
         <v>14.7586480006429</v>
       </c>
     </row>
-    <row r="446" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A446" s="4">
         <v>444</v>
       </c>
@@ -37414,7 +37405,7 @@
         <v>14.951896562116101</v>
       </c>
     </row>
-    <row r="447" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A447" s="4">
         <v>445</v>
       </c>
@@ -37496,7 +37487,7 @@
         <v>15.5170034839955</v>
       </c>
     </row>
-    <row r="448" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A448" s="4">
         <v>446</v>
       </c>
@@ -37578,7 +37569,7 @@
         <v>17.431205146225601</v>
       </c>
     </row>
-    <row r="449" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A449" s="4">
         <v>447</v>
       </c>
@@ -37660,7 +37651,7 @@
         <v>19.1206474373075</v>
       </c>
     </row>
-    <row r="450" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A450" s="4">
         <v>448</v>
       </c>
@@ -37742,7 +37733,7 @@
         <v>20.7295214615167</v>
       </c>
     </row>
-    <row r="451" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A451" s="4">
         <v>449</v>
       </c>
@@ -37824,7 +37815,7 @@
         <v>21.8309555281553</v>
       </c>
     </row>
-    <row r="452" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A452" s="4">
         <v>450</v>
       </c>
@@ -37906,7 +37897,7 @@
         <v>21.9815681323878</v>
       </c>
     </row>
-    <row r="453" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A453" s="4">
         <v>451</v>
       </c>
@@ -37988,7 +37979,7 @@
         <v>21.994878157898899</v>
       </c>
     </row>
-    <row r="454" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A454" s="4">
         <v>452</v>
       </c>
@@ -38070,7 +38061,7 @@
         <v>22.736988437650801</v>
       </c>
     </row>
-    <row r="455" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A455" s="4">
         <v>453</v>
       </c>
@@ -38152,7 +38143,7 @@
         <v>23.426090840277599</v>
       </c>
     </row>
-    <row r="456" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A456" s="4">
         <v>454</v>
       </c>
@@ -38234,7 +38225,7 @@
         <v>24.3922916910028</v>
       </c>
     </row>
-    <row r="457" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A457" s="4">
         <v>455</v>
       </c>
@@ -38316,7 +38307,7 @@
         <v>25.052390563449102</v>
       </c>
     </row>
-    <row r="458" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A458" s="4">
         <v>456</v>
       </c>
@@ -38398,7 +38389,7 @@
         <v>26.2077623299962</v>
       </c>
     </row>
-    <row r="459" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A459" s="4">
         <v>457</v>
       </c>
@@ -38480,7 +38471,7 @@
         <v>27.435884325085102</v>
       </c>
     </row>
-    <row r="460" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A460" s="4">
         <v>458</v>
       </c>
@@ -38562,7 +38553,7 @@
         <v>28.5370556655485</v>
       </c>
     </row>
-    <row r="461" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A461" s="4">
         <v>459</v>
       </c>
@@ -38644,7 +38635,7 @@
         <v>30.907045423627299</v>
       </c>
     </row>
-    <row r="462" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A462" s="4">
         <v>460</v>
       </c>
@@ -38726,7 +38717,7 @@
         <v>33.586863040948401</v>
       </c>
     </row>
-    <row r="463" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A463" s="4">
         <v>461</v>
       </c>
@@ -38808,7 +38799,7 @@
         <v>35.035803606518698</v>
       </c>
     </row>
-    <row r="464" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A464" s="4">
         <v>462</v>
       </c>
@@ -38890,7 +38881,7 @@
         <v>36.293336032319701</v>
       </c>
     </row>
-    <row r="465" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="465" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A465" s="4">
         <v>463</v>
       </c>
@@ -38972,7 +38963,7 @@
         <v>36.319274648816197</v>
       </c>
     </row>
-    <row r="466" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A466" s="4">
         <v>464</v>
       </c>
@@ -39054,7 +39045,7 @@
         <v>36.2749183166666</v>
       </c>
     </row>
-    <row r="467" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A467" s="4">
         <v>465</v>
       </c>
@@ -39136,7 +39127,7 @@
         <v>36.221345245740899</v>
       </c>
     </row>
-    <row r="468" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="468" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A468" s="4">
         <v>466</v>
       </c>
@@ -39218,7 +39209,7 @@
         <v>35.285229299660898</v>
       </c>
     </row>
-    <row r="469" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A469" s="4">
         <v>467</v>
       </c>
@@ -39300,7 +39291,7 @@
         <v>34.491844671828403</v>
       </c>
     </row>
-    <row r="470" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A470" s="4">
         <v>468</v>
       </c>
@@ -39382,7 +39373,7 @@
         <v>34.539741210403903</v>
       </c>
     </row>
-    <row r="471" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A471" s="4">
         <v>469</v>
       </c>
@@ -39464,7 +39455,7 @@
         <v>35.215494782381597</v>
       </c>
     </row>
-    <row r="472" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A472" s="4">
         <v>470</v>
       </c>
@@ -39546,7 +39537,7 @@
         <v>35.912930159901897</v>
       </c>
     </row>
-    <row r="473" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A473" s="4">
         <v>471</v>
       </c>
@@ -39628,7 +39619,7 @@
         <v>36.983497102724797</v>
       </c>
     </row>
-    <row r="474" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A474" s="4">
         <v>472</v>
       </c>
@@ -39710,7 +39701,7 @@
         <v>38.187671721008201</v>
       </c>
     </row>
-    <row r="475" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="475" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A475" s="4">
         <v>473</v>
       </c>
@@ -39792,7 +39783,7 @@
         <v>39.099087402643597</v>
       </c>
     </row>
-    <row r="476" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A476" s="4">
         <v>474</v>
       </c>
@@ -39874,7 +39865,7 @@
         <v>39.172245084957801</v>
       </c>
     </row>
-    <row r="477" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A477" s="4">
         <v>475</v>
       </c>
@@ -39956,7 +39947,7 @@
         <v>39.492990098616197</v>
       </c>
     </row>
-    <row r="478" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A478" s="4">
         <v>476</v>
       </c>
@@ -40038,7 +40029,7 @@
         <v>39.496202088094599</v>
       </c>
     </row>
-    <row r="479" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A479" s="4">
         <v>477</v>
       </c>
@@ -40120,7 +40111,7 @@
         <v>39.624171734112402</v>
       </c>
     </row>
-    <row r="480" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A480" s="4">
         <v>478</v>
       </c>
@@ -40202,7 +40193,7 @@
         <v>38.991812702546298</v>
       </c>
     </row>
-    <row r="481" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A481" s="4">
         <v>479</v>
       </c>
@@ -40284,7 +40275,7 @@
         <v>37.411146186790901</v>
       </c>
     </row>
-    <row r="482" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A482" s="4">
         <v>480</v>
       </c>
@@ -40366,7 +40357,7 @@
         <v>35.048205196674999</v>
       </c>
     </row>
-    <row r="483" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A483" s="4">
         <v>481</v>
       </c>
@@ -40448,7 +40439,7 @@
         <v>33.114286217894701</v>
       </c>
     </row>
-    <row r="484" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="484" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A484" s="4">
         <v>482</v>
       </c>
@@ -40530,7 +40521,7 @@
         <v>31.660245288681502</v>
       </c>
     </row>
-    <row r="485" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="485" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A485" s="4">
         <v>483</v>
       </c>
@@ -40612,7 +40603,7 @@
         <v>30.7003919657691</v>
       </c>
     </row>
-    <row r="486" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="486" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A486" s="4">
         <v>484</v>
       </c>
@@ -40694,7 +40685,7 @@
         <v>30.074803034748701</v>
       </c>
     </row>
-    <row r="487" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="487" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A487" s="4">
         <v>485</v>
       </c>
@@ -40776,7 +40767,7 @@
         <v>30.169507806168099</v>
       </c>
     </row>
-    <row r="488" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="488" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A488" s="4">
         <v>486</v>
       </c>
@@ -40858,7 +40849,7 @@
         <v>29.910825236138699</v>
       </c>
     </row>
-    <row r="489" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="489" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A489" s="4">
         <v>487</v>
       </c>
@@ -40940,7 +40931,7 @@
         <v>30.2008063990999</v>
       </c>
     </row>
-    <row r="490" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="490" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A490" s="4">
         <v>488</v>
       </c>
@@ -41022,7 +41013,7 @@
         <v>30.505063722257201</v>
       </c>
     </row>
-    <row r="491" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="491" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A491" s="4">
         <v>489</v>
       </c>
@@ -41104,7 +41095,7 @@
         <v>30.638516125959701</v>
       </c>
     </row>
-    <row r="492" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="492" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A492" s="4">
         <v>490</v>
       </c>
@@ -41186,7 +41177,7 @@
         <v>30.983166642136901</v>
       </c>
     </row>
-    <row r="493" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="493" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A493" s="4">
         <v>491</v>
       </c>
@@ -41268,7 +41259,7 @@
         <v>31.0967744154316</v>
       </c>
     </row>
-    <row r="494" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="494" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A494" s="4">
         <v>492</v>
       </c>
@@ -41350,7 +41341,7 @@
         <v>31.463819131952899</v>
       </c>
     </row>
-    <row r="495" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="495" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A495" s="4">
         <v>493</v>
       </c>
@@ -41432,7 +41423,7 @@
         <v>30.938772501267199</v>
       </c>
     </row>
-    <row r="496" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="496" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A496" s="4">
         <v>494</v>
       </c>
@@ -41514,7 +41505,7 @@
         <v>30.535927713522199</v>
       </c>
     </row>
-    <row r="497" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="497" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A497" s="4">
         <v>495</v>
       </c>
@@ -41596,7 +41587,7 @@
         <v>30.282776040365199</v>
       </c>
     </row>
-    <row r="498" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="498" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A498" s="4">
         <v>496</v>
       </c>
@@ -41678,7 +41669,7 @@
         <v>30.497836595735201</v>
       </c>
     </row>
-    <row r="499" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="499" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A499" s="4">
         <v>497</v>
       </c>
@@ -41760,7 +41751,7 @@
         <v>30.912779117799101</v>
       </c>
     </row>
-    <row r="500" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="500" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A500" s="4">
         <v>498</v>
       </c>
@@ -41842,7 +41833,7 @@
         <v>31.2099596113381</v>
       </c>
     </row>
-    <row r="501" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="501" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A501" s="4">
         <v>499</v>
       </c>
@@ -41924,7 +41915,7 @@
         <v>31.113824222237</v>
       </c>
     </row>
-    <row r="502" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="502" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A502" s="4">
         <v>500</v>
       </c>
@@ -42006,7 +41997,7 @@
         <v>30.960371035230398</v>
       </c>
     </row>
-    <row r="503" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="503" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A503" s="4">
         <v>501</v>
       </c>
@@ -42054,7 +42045,7 @@
         <f>100*testdata[[#This Row],[-DM14]]/testdata[[#This Row],[TR14]]</f>
         <v>31.150968674636061</v>
       </c>
-      <c r="N503" s="6">
+      <c r="N503" s="11">
         <f>100*ABS(testdata[[#This Row],[+DI14]]-testdata[[#This Row],[-DI14]])/(testdata[[#This Row],[+DI14]]+testdata[[#This Row],[-DI14]])</f>
         <v>27.387308306629919</v>
       </c>

</xml_diff>